<commit_message>
Corrections suite aux revues 75aebc17afdcf6c5f655e235258d83bc2e6ad34d
</commit_message>
<xml_diff>
--- a/htr-strucGenerale-CDA/ig/StructureDefinition-Auteur.xlsx
+++ b/htr-strucGenerale-CDA/ig/StructureDefinition-Auteur.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-18T10:35:11+00:00</t>
+    <t>2025-04-18T14:53:38+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -235,7 +235,7 @@
     <t/>
   </si>
   <si>
-    <t>0</t>
+    <t>1</t>
   </si>
   <si>
     <t>*</t>
@@ -248,10 +248,10 @@
     <t>Base</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>Auteur.roleFonctionnel</t>
-  </si>
-  <si>
-    <t>1</t>
   </si>
   <si>
     <t xml:space="preserve">CodeableConcept
@@ -275,7 +275,7 @@
   </si>
   <si>
     <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PersonneStructureAuteur
-https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/Systeme</t>
+https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/SystemeStructureAuteur</t>
   </si>
   <si>
     <t>Auteur du document : ce peut être un professionnel, un patient/usager ou un système. Pour un professionnel ou un système, la structure de rattachement doit être précisée.</t>
@@ -818,7 +818,7 @@
         <v>76</v>
       </c>
       <c r="AG2" t="s" s="2">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="AH2" t="s" s="2">
         <v>74</v>
@@ -832,10 +832,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" t="s" s="2">
@@ -843,10 +843,10 @@
       </c>
       <c r="E3" s="2"/>
       <c r="F3" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G3" t="s" s="2">
         <v>73</v>
-      </c>
-      <c r="G3" t="s" s="2">
-        <v>78</v>
       </c>
       <c r="H3" t="s" s="2">
         <v>72</v>
@@ -915,13 +915,13 @@
         <v>72</v>
       </c>
       <c r="AF3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AG3" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="AG3" t="s" s="2">
+      <c r="AH3" t="s" s="2">
         <v>73</v>
-      </c>
-      <c r="AH3" t="s" s="2">
-        <v>78</v>
       </c>
       <c r="AI3" t="s" s="2">
         <v>72</v>
@@ -943,10 +943,10 @@
       </c>
       <c r="E4" s="2"/>
       <c r="F4" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="G4" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H4" t="s" s="2">
         <v>72</v>
@@ -1018,10 +1018,10 @@
         <v>81</v>
       </c>
       <c r="AG4" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH4" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AI4" t="s" s="2">
         <v>72</v>
@@ -1043,10 +1043,10 @@
       </c>
       <c r="E5" s="2"/>
       <c r="F5" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H5" t="s" s="2">
         <v>72</v>
@@ -1118,10 +1118,10 @@
         <v>84</v>
       </c>
       <c r="AG5" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH5" t="s" s="2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AI5" t="s" s="2">
         <v>72</v>

</xml_diff>